<commit_message>
feat: Add Item unified dialog + template refresh with non-DB data
- Replace 'Add SKU' + 'Add Material' buttons with single 'Add Item'
- AddItemDialog: EntityType combo (SKU/MATERIAL) at top, common fields below
  * Allow Grouping row visible only when SKU selected
  * Label/hint text updates dynamically on type switch
- templates/: all sample files now contain codes NOT in the current DB
  * 01_Item_Master.xlsx — SKU-E10, SKU-E30, SKU-F05, MAT-010, MAT-011
  * 03_Room_Process_Master.xlsx — ROOM-G, ROOM-H (new rooms)
  * 04_Process_Routing.xlsx — routing for new SKUs/Materials above
  * 05_Sales_Order.xlsx — SO-2026-020~023 (new SO numbers)
  * 07_Inventory.xlsx — LOT-2026-NEW-001~003 (new lot numbers)
- Removed legacy 01_SKU_Master.xlsx and 02_Material_Master.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/01_Item_Master.xlsx
+++ b/templates/01_Item_Master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -482,24 +482,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SKU-A10</t>
+          <t>SKU-E10</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Product A 10pcs/box</t>
+          <t>Product E 10pcs/box</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>New line</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -509,26 +513,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SKU-A30</t>
+          <t>SKU-E30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Product A 30pcs/box</t>
+          <t>Product E 30pcs/box</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>30</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>QC 7 days</t>
+          <t>Individual planning</t>
         </is>
       </c>
     </row>
@@ -540,216 +544,98 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SKU-B04</t>
+          <t>SKU-F05</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Product B 4pcs/box</t>
+          <t>Product F 5pcs/pack</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Clinic pack</t>
+          <t>Stability 7d</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>MATERIAL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SKU-B25</t>
+          <t>MAT-010</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Product B 25pcs/box</t>
+          <t>Semi-fin X (tablet)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>QC 2 days</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>MATERIAL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SKU-C30</t>
+          <t>MAT-011</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Product C 30pcs/box</t>
+          <t>Semi-fin Y (capsule)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Stability QC 14 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>SKU-D01</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Product D single unit</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Bulk</t>
+          <t>No QC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MATERIAL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MAT-001</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Semi-fin A (granule)</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>QC 1 day</t>
+          <t># EntityType: SKU or MATERIAL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MATERIAL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>MAT-002</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Semi-fin B (solution)</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Sterility QC 3 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MATERIAL</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MAT-003</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Semi-fin C (conc.)</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>No QC</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t># EntityType: SKU or MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t># AllowGrouping: 1=batch same-SKU orders, 0=plan each order individually (SKU only)</t>
+          <t># AllowGrouping: 1=batch same-SKU orders, 0=plan individually (SKU only)</t>
         </is>
       </c>
     </row>

</xml_diff>